<commit_message>
Enhance testing framework with new shift and RBAC management features
- Added new test commands for shift management and RBAC role creation in package.json.
- Updated README.md to include instructions for new test commands and CI configurations.
- Introduced new page objects and handlers for managing shifts and RBAC roles, improving test organization and maintainability.
- Enhanced existing test cases to automate RBAC role creation and shift management scenarios.
- Increased timeout for GitHub Actions E2E job to accommodate longer test execution times.
- Updated JSON test data to reflect new automated test cases and adjusted priority levels for better test management.
</commit_message>
<xml_diff>
--- a/e2e/data/catalogs/rbac-create-role.xlsx
+++ b/e2e/data/catalogs/rbac-create-role.xlsx
@@ -64,70 +64,70 @@
     <t>Open /rbac-management/create-role; title Create Role; Save disabled until name, description, and at least one permission</t>
   </si>
   <si>
+    <t>P0</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>RBAC-UI-02</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>User:Read All</t>
+  </si>
+  <si>
+    <t>User:Read+Read All</t>
+  </si>
+  <si>
+    <t>Empty role name shows Role name is required; save stays disabled</t>
+  </si>
+  <si>
+    <t>RBAC-UI-03</t>
+  </si>
+  <si>
+    <t>auto_no_perm</t>
+  </si>
+  <si>
+    <t>Empty description shows Description is required; save stays disabled</t>
+  </si>
+  <si>
+    <t>RBAC-UI-04</t>
+  </si>
+  <si>
+    <t>no permissions selected</t>
+  </si>
+  <si>
+    <t>Save with zero permissions shows At least one permission must be selected</t>
+  </si>
+  <si>
+    <t>RBAC-ROLE-001</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+  <si>
+    <t>auto_rbac_001_user_create</t>
+  </si>
+  <si>
+    <t>User Management only: click User Create; assert dependencyRules auto-selects</t>
+  </si>
+  <si>
+    <t>User:Create</t>
+  </si>
+  <si>
+    <t>Role:Read|Shift:Read|User:Activate Or Deactivate+Assign All/Unassign All+Assign/Unassign+Create+Read</t>
+  </si>
+  <si>
+    <t>Role is created; list shows the new role; selected permissions include dependencyRules auto-grants</t>
+  </si>
+  <si>
     <t>P2</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Not automated yet</t>
-  </si>
-  <si>
-    <t>RBAC-UI-02</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>User:Read All</t>
-  </si>
-  <si>
-    <t>User:Read+Read All</t>
-  </si>
-  <si>
-    <t>Empty role name shows Role name is required; save stays disabled</t>
-  </si>
-  <si>
-    <t>RBAC-UI-03</t>
-  </si>
-  <si>
-    <t>auto_no_perm</t>
-  </si>
-  <si>
-    <t>Empty description shows Description is required; save stays disabled</t>
-  </si>
-  <si>
-    <t>RBAC-UI-04</t>
-  </si>
-  <si>
-    <t>no permissions selected</t>
-  </si>
-  <si>
-    <t>Save with zero permissions shows At least one permission must be selected</t>
-  </si>
-  <si>
-    <t>RBAC-ROLE-001</t>
-  </si>
-  <si>
-    <t>user</t>
-  </si>
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>auto_rbac_001_user_create</t>
-  </si>
-  <si>
-    <t>User Management only: click User Create; assert dependencyRules auto-selects</t>
-  </si>
-  <si>
-    <t>User:Create</t>
-  </si>
-  <si>
-    <t>Role:Read|Shift:Read|User:Activate Or Deactivate+Assign All/Unassign All+Assign/Unassign+Create+Read</t>
-  </si>
-  <si>
-    <t>Role is created; list shows the new role; selected permissions include dependencyRules auto-grants</t>
   </si>
   <si>
     <t>RBAC-ROLE-002</t>
@@ -1685,7 +1685,7 @@
         <v>18</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>15</v>
@@ -1693,7 +1693,7 @@
     </row>
     <row r="3" ht="48" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>13</v>
@@ -1705,16 +1705,16 @@
         <v>15</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>17</v>
@@ -1723,7 +1723,7 @@
         <v>18</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>15</v>
@@ -1731,7 +1731,7 @@
     </row>
     <row r="4" ht="48" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>13</v>
@@ -1740,19 +1740,19 @@
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>17</v>
@@ -1761,7 +1761,7 @@
         <v>18</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>15</v>
@@ -1769,7 +1769,7 @@
     </row>
     <row r="5" ht="48" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>13</v>
@@ -1778,19 +1778,19 @@
         <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>17</v>
@@ -1799,7 +1799,7 @@
         <v>18</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>15</v>
@@ -1807,37 +1807,37 @@
     </row>
     <row r="6" ht="48" customHeight="1" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="C6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>37</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>15</v>
@@ -1848,10 +1848,10 @@
         <v>39</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>40</v>
@@ -1860,22 +1860,22 @@
         <v>41</v>
       </c>
       <c r="F7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="H7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>15</v>
@@ -1886,10 +1886,10 @@
         <v>42</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>43</v>
@@ -1904,16 +1904,16 @@
         <v>46</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>15</v>
@@ -1927,7 +1927,7 @@
         <v>48</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>49</v>
@@ -1942,16 +1942,16 @@
         <v>52</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>15</v>
@@ -1965,7 +1965,7 @@
         <v>48</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>54</v>
@@ -1980,16 +1980,16 @@
         <v>57</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>15</v>
@@ -2003,7 +2003,7 @@
         <v>48</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>59</v>
@@ -2018,16 +2018,16 @@
         <v>62</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>15</v>
@@ -2041,7 +2041,7 @@
         <v>48</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>64</v>
@@ -2056,16 +2056,16 @@
         <v>67</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>15</v>
@@ -2079,7 +2079,7 @@
         <v>48</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>69</v>
@@ -2094,16 +2094,16 @@
         <v>72</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>15</v>
@@ -2117,7 +2117,7 @@
         <v>48</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>74</v>
@@ -2132,16 +2132,16 @@
         <v>77</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>15</v>
@@ -2155,7 +2155,7 @@
         <v>48</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>79</v>
@@ -2170,16 +2170,16 @@
         <v>82</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>15</v>
@@ -2193,7 +2193,7 @@
         <v>48</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>84</v>
@@ -2208,16 +2208,16 @@
         <v>87</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>15</v>
@@ -2231,7 +2231,7 @@
         <v>48</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>89</v>
@@ -2246,16 +2246,16 @@
         <v>92</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>15</v>
@@ -2269,7 +2269,7 @@
         <v>48</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>94</v>
@@ -2284,16 +2284,16 @@
         <v>97</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>15</v>
@@ -2307,7 +2307,7 @@
         <v>48</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>99</v>
@@ -2322,16 +2322,16 @@
         <v>102</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>15</v>
@@ -2345,7 +2345,7 @@
         <v>48</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>104</v>
@@ -2360,16 +2360,16 @@
         <v>107</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>15</v>
@@ -2383,7 +2383,7 @@
         <v>48</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>109</v>
@@ -2398,16 +2398,16 @@
         <v>82</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>15</v>
@@ -2421,7 +2421,7 @@
         <v>48</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>113</v>
@@ -2436,16 +2436,16 @@
         <v>116</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>15</v>
@@ -2459,7 +2459,7 @@
         <v>118</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>119</v>
@@ -2474,16 +2474,16 @@
         <v>122</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>15</v>
@@ -2497,7 +2497,7 @@
         <v>118</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>124</v>
@@ -2512,16 +2512,16 @@
         <v>127</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>15</v>
@@ -2535,7 +2535,7 @@
         <v>118</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>129</v>
@@ -2550,16 +2550,16 @@
         <v>132</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J25" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>15</v>
@@ -2573,7 +2573,7 @@
         <v>118</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>134</v>
@@ -2588,16 +2588,16 @@
         <v>137</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>15</v>
@@ -2611,7 +2611,7 @@
         <v>118</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>139</v>
@@ -2626,16 +2626,16 @@
         <v>142</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>15</v>
@@ -2649,7 +2649,7 @@
         <v>118</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>144</v>
@@ -2664,16 +2664,16 @@
         <v>147</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>15</v>
@@ -2687,7 +2687,7 @@
         <v>118</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>149</v>
@@ -2702,16 +2702,16 @@
         <v>152</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J29" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>15</v>
@@ -2725,7 +2725,7 @@
         <v>118</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>154</v>
@@ -2740,16 +2740,16 @@
         <v>157</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J30" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>15</v>
@@ -2763,7 +2763,7 @@
         <v>118</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>159</v>
@@ -2778,16 +2778,16 @@
         <v>162</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>15</v>
@@ -2801,7 +2801,7 @@
         <v>118</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>164</v>
@@ -2816,16 +2816,16 @@
         <v>167</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>15</v>
@@ -2839,7 +2839,7 @@
         <v>118</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>169</v>
@@ -2854,16 +2854,16 @@
         <v>172</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J33" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>15</v>
@@ -2877,7 +2877,7 @@
         <v>118</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>174</v>
@@ -2892,16 +2892,16 @@
         <v>177</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>15</v>
@@ -2915,7 +2915,7 @@
         <v>118</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>179</v>
@@ -2930,16 +2930,16 @@
         <v>152</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>15</v>
@@ -2953,7 +2953,7 @@
         <v>118</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>183</v>
@@ -2968,16 +2968,16 @@
         <v>186</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>15</v>
@@ -2991,7 +2991,7 @@
         <v>118</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>188</v>
@@ -3006,16 +3006,16 @@
         <v>191</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>15</v>
@@ -3029,7 +3029,7 @@
         <v>118</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>193</v>
@@ -3044,16 +3044,16 @@
         <v>196</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L38" s="2" t="s">
         <v>15</v>
@@ -3067,7 +3067,7 @@
         <v>118</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>198</v>
@@ -3082,16 +3082,16 @@
         <v>201</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>15</v>
@@ -3105,7 +3105,7 @@
         <v>118</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>203</v>
@@ -3120,16 +3120,16 @@
         <v>206</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>15</v>
@@ -3143,7 +3143,7 @@
         <v>118</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>208</v>
@@ -3158,16 +3158,16 @@
         <v>211</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>15</v>
@@ -3181,7 +3181,7 @@
         <v>118</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>213</v>
@@ -3196,16 +3196,16 @@
         <v>216</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>15</v>
@@ -3219,7 +3219,7 @@
         <v>118</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>218</v>
@@ -3234,16 +3234,16 @@
         <v>221</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J43" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>15</v>
@@ -3257,7 +3257,7 @@
         <v>118</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>223</v>
@@ -3272,16 +3272,16 @@
         <v>226</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>15</v>
@@ -3295,7 +3295,7 @@
         <v>118</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>228</v>
@@ -3310,16 +3310,16 @@
         <v>231</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>15</v>
@@ -3333,7 +3333,7 @@
         <v>118</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>233</v>
@@ -3348,16 +3348,16 @@
         <v>236</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J46" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K46" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>15</v>
@@ -3371,7 +3371,7 @@
         <v>118</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>238</v>
@@ -3386,16 +3386,16 @@
         <v>241</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J47" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K47" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>15</v>
@@ -3409,7 +3409,7 @@
         <v>118</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>243</v>
@@ -3424,16 +3424,16 @@
         <v>246</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J48" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>15</v>
@@ -3447,7 +3447,7 @@
         <v>118</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>248</v>
@@ -3462,16 +3462,16 @@
         <v>221</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>15</v>
@@ -3485,7 +3485,7 @@
         <v>118</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>252</v>
@@ -3500,16 +3500,16 @@
         <v>255</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J50" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>15</v>
@@ -3523,7 +3523,7 @@
         <v>118</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>257</v>
@@ -3538,16 +3538,16 @@
         <v>260</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J51" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K51" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>15</v>
@@ -3561,7 +3561,7 @@
         <v>118</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>262</v>
@@ -3576,16 +3576,16 @@
         <v>265</v>
       </c>
       <c r="H52" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J52" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K52" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>15</v>
@@ -3599,7 +3599,7 @@
         <v>118</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>267</v>
@@ -3614,16 +3614,16 @@
         <v>270</v>
       </c>
       <c r="H53" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>15</v>
@@ -3637,7 +3637,7 @@
         <v>118</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>272</v>
@@ -3652,16 +3652,16 @@
         <v>275</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J54" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K54" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L54" s="2" t="s">
         <v>15</v>
@@ -3675,7 +3675,7 @@
         <v>118</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>277</v>
@@ -3690,16 +3690,16 @@
         <v>280</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J55" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K55" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L55" s="2" t="s">
         <v>15</v>
@@ -3713,7 +3713,7 @@
         <v>118</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>282</v>
@@ -3728,16 +3728,16 @@
         <v>285</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J56" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>15</v>
@@ -3751,7 +3751,7 @@
         <v>118</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>287</v>
@@ -3766,16 +3766,16 @@
         <v>290</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J57" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K57" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L57" s="2" t="s">
         <v>15</v>
@@ -3789,7 +3789,7 @@
         <v>118</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>292</v>
@@ -3804,16 +3804,16 @@
         <v>295</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J58" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K58" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L58" s="2" t="s">
         <v>15</v>
@@ -3827,7 +3827,7 @@
         <v>118</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>297</v>
@@ -3842,16 +3842,16 @@
         <v>300</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J59" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>15</v>
@@ -3865,7 +3865,7 @@
         <v>118</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>302</v>
@@ -3880,16 +3880,16 @@
         <v>305</v>
       </c>
       <c r="H60" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I60" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J60" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L60" s="2" t="s">
         <v>15</v>
@@ -3903,7 +3903,7 @@
         <v>118</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>307</v>
@@ -3918,16 +3918,16 @@
         <v>310</v>
       </c>
       <c r="H61" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I61" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J61" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L61" s="2" t="s">
         <v>15</v>
@@ -3941,7 +3941,7 @@
         <v>118</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>312</v>
@@ -3956,16 +3956,16 @@
         <v>315</v>
       </c>
       <c r="H62" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J62" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K62" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L62" s="2" t="s">
         <v>15</v>
@@ -3979,7 +3979,7 @@
         <v>118</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>317</v>
@@ -3994,16 +3994,16 @@
         <v>290</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I63" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J63" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K63" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L63" s="2" t="s">
         <v>15</v>
@@ -4017,7 +4017,7 @@
         <v>118</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>321</v>
@@ -4032,16 +4032,16 @@
         <v>324</v>
       </c>
       <c r="H64" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J64" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K64" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>15</v>
@@ -4055,7 +4055,7 @@
         <v>326</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>327</v>
@@ -4070,16 +4070,16 @@
         <v>330</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>15</v>
@@ -4093,7 +4093,7 @@
         <v>326</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>332</v>
@@ -4108,16 +4108,16 @@
         <v>335</v>
       </c>
       <c r="H66" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J66" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K66" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>15</v>
@@ -4131,7 +4131,7 @@
         <v>326</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>337</v>
@@ -4146,16 +4146,16 @@
         <v>340</v>
       </c>
       <c r="H67" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I67" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>15</v>
@@ -4169,7 +4169,7 @@
         <v>326</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>342</v>
@@ -4184,16 +4184,16 @@
         <v>345</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I68" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L68" s="2" t="s">
         <v>15</v>
@@ -4207,7 +4207,7 @@
         <v>326</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>347</v>
@@ -4222,16 +4222,16 @@
         <v>350</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I69" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J69" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>15</v>
@@ -4245,7 +4245,7 @@
         <v>326</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>352</v>
@@ -4260,16 +4260,16 @@
         <v>355</v>
       </c>
       <c r="H70" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I70" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>15</v>
@@ -4283,7 +4283,7 @@
         <v>326</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>357</v>
@@ -4298,16 +4298,16 @@
         <v>360</v>
       </c>
       <c r="H71" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I71" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J71" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L71" s="2" t="s">
         <v>15</v>
@@ -4321,7 +4321,7 @@
         <v>326</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>362</v>
@@ -4336,16 +4336,16 @@
         <v>365</v>
       </c>
       <c r="H72" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I72" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L72" s="2" t="s">
         <v>15</v>
@@ -4359,7 +4359,7 @@
         <v>326</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>367</v>
@@ -4374,16 +4374,16 @@
         <v>370</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I73" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L73" s="2" t="s">
         <v>15</v>
@@ -4397,7 +4397,7 @@
         <v>326</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>372</v>
@@ -4412,16 +4412,16 @@
         <v>375</v>
       </c>
       <c r="H74" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I74" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K74" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L74" s="2" t="s">
         <v>15</v>
@@ -4435,7 +4435,7 @@
         <v>326</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>377</v>
@@ -4450,16 +4450,16 @@
         <v>380</v>
       </c>
       <c r="H75" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I75" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J75" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>15</v>
@@ -4473,7 +4473,7 @@
         <v>326</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>382</v>
@@ -4488,16 +4488,16 @@
         <v>385</v>
       </c>
       <c r="H76" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I76" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L76" s="2" t="s">
         <v>15</v>
@@ -4511,7 +4511,7 @@
         <v>326</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>387</v>
@@ -4526,16 +4526,16 @@
         <v>390</v>
       </c>
       <c r="H77" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I77" s="2" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="J77" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K77" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="L77" s="2" t="s">
         <v>15</v>

</xml_diff>